<commit_message>
working on common bug fixing...
</commit_message>
<xml_diff>
--- a/Sync/Documents/FujiSync4D.Issues_03292012.xlsx
+++ b/Sync/Documents/FujiSync4D.Issues_03292012.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9302"/>
   <workbookPr defaultThemeVersion="124226"/>
   <bookViews>
-    <workbookView xWindow="120" yWindow="30" windowWidth="15195" windowHeight="11760" activeTab="1"/>
+    <workbookView xWindow="120" yWindow="30" windowWidth="15195" windowHeight="11760"/>
   </bookViews>
   <sheets>
     <sheet name="03292012" sheetId="1" r:id="rId1"/>
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="86" uniqueCount="47">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="87" uniqueCount="45">
   <si>
     <t>Sr.No</t>
   </si>
@@ -483,18 +483,9 @@
     <t>Please change footer of website as shown in mockup website</t>
   </si>
   <si>
-    <t>InProgress</t>
-  </si>
-  <si>
     <t>Done</t>
   </si>
   <si>
-    <t>Question To Ask</t>
-  </si>
-  <si>
-    <t>Partially Done</t>
-  </si>
-  <si>
     <t>Related to TaskNo. 7</t>
   </si>
   <si>
@@ -1135,6 +1126,9 @@
   </si>
   <si>
     <t>General</t>
+  </si>
+  <si>
+    <t>In Progress</t>
   </si>
 </sst>
 </file>
@@ -1570,16 +1564,16 @@
         <v>1</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="D1" s="2" t="s">
         <v>2</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="F1" s="3" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
     </row>
     <row r="2" spans="1:6" ht="30" x14ac:dyDescent="0.25">
@@ -1590,10 +1584,10 @@
         <v>3</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="D2" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="3" spans="1:6" ht="30" x14ac:dyDescent="0.25">
@@ -1604,10 +1598,10 @@
         <v>4</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="D3" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="4" spans="1:6" ht="45" x14ac:dyDescent="0.25">
@@ -1618,10 +1612,10 @@
         <v>5</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="D4" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="5" spans="1:6" s="4" customFormat="1" ht="30" x14ac:dyDescent="0.25">
@@ -1629,19 +1623,19 @@
         <v>4</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E5" s="4" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="F5" s="4" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
     </row>
     <row r="6" spans="1:6" ht="30" x14ac:dyDescent="0.25">
@@ -1652,10 +1646,10 @@
         <v>6</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="D6" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="7" spans="1:6" ht="45" x14ac:dyDescent="0.25">
@@ -1666,10 +1660,10 @@
         <v>7</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="D7" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="8" spans="1:6" ht="135" x14ac:dyDescent="0.25">
@@ -1680,10 +1674,10 @@
         <v>8</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="D8" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
     </row>
     <row r="9" spans="1:6" ht="30" x14ac:dyDescent="0.25">
@@ -1694,7 +1688,7 @@
         <v>9</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="D9" t="s">
         <v>15</v>
@@ -1708,13 +1702,13 @@
         <v>10</v>
       </c>
       <c r="C10" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="D10" t="s">
         <v>44</v>
       </c>
-      <c r="D10" t="s">
-        <v>18</v>
-      </c>
       <c r="E10" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
     </row>
     <row r="11" spans="1:6" ht="75" x14ac:dyDescent="0.25">
@@ -1725,13 +1719,13 @@
         <v>11</v>
       </c>
       <c r="C11" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="D11" t="s">
         <v>44</v>
       </c>
-      <c r="D11" t="s">
+      <c r="E11" t="s">
         <v>21</v>
-      </c>
-      <c r="E11" t="s">
-        <v>24</v>
       </c>
     </row>
     <row r="12" spans="1:6" s="4" customFormat="1" ht="30" x14ac:dyDescent="0.25">
@@ -1739,19 +1733,19 @@
         <v>11</v>
       </c>
       <c r="B12" s="5" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="D12" s="4" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="E12" s="4" t="s">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="F12" s="4" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
     </row>
     <row r="13" spans="1:6" ht="45" x14ac:dyDescent="0.25">
@@ -1762,10 +1756,10 @@
         <v>12</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="D13" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="14" spans="1:6" ht="60" x14ac:dyDescent="0.25">
@@ -1776,10 +1770,10 @@
         <v>13</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="D14" t="s">
-        <v>21</v>
+        <v>15</v>
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.25">
@@ -1790,10 +1784,10 @@
         <v>14</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="D15" t="s">
-        <v>21</v>
+        <v>15</v>
       </c>
     </row>
   </sheetData>
@@ -1809,6 +1803,7 @@
   <cols>
     <col min="2" max="2" width="104.140625" customWidth="1"/>
     <col min="3" max="3" width="17.28515625" customWidth="1"/>
+    <col min="4" max="4" width="10.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -1819,16 +1814,16 @@
         <v>1</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="D1" s="2" t="s">
         <v>2</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="F1" s="3" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
     </row>
     <row r="2" spans="1:6" ht="45" x14ac:dyDescent="0.25">
@@ -1836,10 +1831,10 @@
         <v>1</v>
       </c>
       <c r="B2" s="6" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="C2" s="6" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
     </row>
     <row r="3" spans="1:6" ht="45" x14ac:dyDescent="0.25">
@@ -1847,10 +1842,10 @@
         <v>2</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="C3" s="6" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
@@ -1858,10 +1853,10 @@
         <v>3</v>
       </c>
       <c r="B4" s="7" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
     </row>
     <row r="5" spans="1:6" ht="30" x14ac:dyDescent="0.25">
@@ -1869,10 +1864,10 @@
         <v>4</v>
       </c>
       <c r="B5" s="7" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
     </row>
     <row r="6" spans="1:6" ht="60" x14ac:dyDescent="0.25">
@@ -1880,10 +1875,10 @@
         <v>5</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="C6" s="6" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
     </row>
     <row r="7" spans="1:6" ht="62.25" x14ac:dyDescent="0.25">
@@ -1891,10 +1886,10 @@
         <v>6</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="C7" s="6" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.25">
@@ -1902,10 +1897,10 @@
         <v>7</v>
       </c>
       <c r="B8" s="8" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="C8" s="6" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
     </row>
     <row r="9" spans="1:6" ht="45" x14ac:dyDescent="0.25">
@@ -1913,10 +1908,13 @@
         <v>8</v>
       </c>
       <c r="B9" s="7" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="C9" s="7" t="s">
-        <v>45</v>
+        <v>42</v>
+      </c>
+      <c r="D9" s="7" t="s">
+        <v>44</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.25">
@@ -1924,10 +1922,10 @@
         <v>9</v>
       </c>
       <c r="B10" s="7" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="C10" s="7" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
     </row>
     <row r="11" spans="1:6" ht="30" x14ac:dyDescent="0.25">
@@ -1935,10 +1933,10 @@
         <v>10</v>
       </c>
       <c r="B11" s="7" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="C11" s="7" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.25">
@@ -1946,10 +1944,10 @@
         <v>11</v>
       </c>
       <c r="B12" s="8" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="C12" s="7" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
     </row>
     <row r="13" spans="1:6" ht="60" x14ac:dyDescent="0.25">
@@ -1957,10 +1955,10 @@
         <v>12</v>
       </c>
       <c r="B13" s="7" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="C13" s="7" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.25">
@@ -1968,10 +1966,10 @@
         <v>13</v>
       </c>
       <c r="B14" s="8" t="s">
+        <v>39</v>
+      </c>
+      <c r="C14" s="7" t="s">
         <v>42</v>
-      </c>
-      <c r="C14" s="7" t="s">
-        <v>45</v>
       </c>
     </row>
   </sheetData>

</xml_diff>